<commit_message>
Add all 4 Tesla listings from search to spreadsheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017jfPwVxZPc8HYePdfQgeuD
</commit_message>
<xml_diff>
--- a/tesla_listings.xlsx
+++ b/tesla_listings.xlsx
@@ -417,8 +417,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="19" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -473,70 +502,85 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>cash_incentive</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>original_down_payment</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>purchase_option</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>months_remaining</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>original_term_months</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>lease_expiry</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>odometer_km</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>km_allowance_total</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>km_per_year</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>free_km_per_year</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>excess_km_charge</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>interest_rate</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>takeover_cash</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>lease_expiry</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>leasing_company</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>exterior</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>interior</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>winter_tires</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>seller</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>seller_phone</t>
         </is>
@@ -545,100 +589,403 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>592758</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.leasebusters.com/details/592758/2024-Tesla-Model%20Y</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Model Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Long Range AWD</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Mont Royal, QC</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>888</v>
+      </c>
+      <c r="I2" t="n">
+        <v>887.5700000000001</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1020.48</v>
+      </c>
+      <c r="L2" t="n">
+        <v>250</v>
+      </c>
+      <c r="M2" t="n">
+        <v>36124.4</v>
+      </c>
+      <c r="N2" t="n">
+        <v>18</v>
+      </c>
+      <c r="O2" t="n">
+        <v>48</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2028-04-08</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>32773</v>
+      </c>
+      <c r="R2" t="n">
+        <v>80000</v>
+      </c>
+      <c r="S2" t="n">
+        <v>31484</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.0626</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Dark Grey</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Francois Domingue</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>(514) 827-7966</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>613254</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>https://www.leasebusters.com/details/613254/2026-Tesla-Model%20Y</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C3" t="n">
         <v>2026</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Tesla</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Model Y</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Long Range AWD</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Mont-Royal, QC</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="H3" t="n">
         <v>971</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I3" t="n">
         <v>970.72</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J3" t="n">
         <v>1116.09</v>
       </c>
-      <c r="K2" t="n">
+      <c r="N3" t="n">
         <v>44</v>
       </c>
-      <c r="L2" t="n">
+      <c r="O3" t="n">
         <v>48</v>
       </c>
-      <c r="M2" t="n">
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2030-06-11</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
         <v>5000</v>
       </c>
-      <c r="N2" t="n">
+      <c r="R3" t="n">
         <v>100000</v>
       </c>
-      <c r="O2" t="n">
+      <c r="S3" t="n">
         <v>25909</v>
       </c>
-      <c r="P2" t="n">
+      <c r="T3" t="n">
         <v>0.15</v>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>3.45%</t>
-        </is>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>2030-06-11</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="U3" t="n">
+        <v>0.0345</v>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>Tesla Motors Canada ULC</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>Dark Grey</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>Black</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
         <is>
           <t>Alexis Auch</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>(438) 929-1891</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>598606</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.leasebusters.com/details/598606/2024-Tesla-Model%20Y</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Model Y</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Long Range AWD</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Blainville, QC</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>1003</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1003.14</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1072.25</v>
+      </c>
+      <c r="N4" t="n">
+        <v>15</v>
+      </c>
+      <c r="O4" t="n">
+        <v>48</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2028-01-09</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>58000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>100000</v>
+      </c>
+      <c r="S4" t="n">
+        <v>33600</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Tesla Motors Canada ULC</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Xavier Clément</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>(438) 464-1254</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>602944</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.leasebusters.com/details/602944/2024-Tesla-Model%20Y</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Model Y</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>RWD</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Richmond Hill, ON</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>713</v>
+      </c>
+      <c r="I5" t="n">
+        <v>813</v>
+      </c>
+      <c r="J5" t="n">
+        <v>935.49</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="N5" t="n">
+        <v>15</v>
+      </c>
+      <c r="O5" t="n">
+        <v>48</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2028-02-03</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>92400</v>
+      </c>
+      <c r="R5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="S5" t="n">
+        <v>6080</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Tesla Finance</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Mohammed A.</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>(647) 280-2531</t>
         </is>
       </c>
     </row>

</xml_diff>